<commit_message>
build(v0.8): regenerate tape-aware release docs
</commit_message>
<xml_diff>
--- a/exports/final/bom/BOM.xlsx
+++ b/exports/final/bom/BOM.xlsx
@@ -13557,12 +13557,12 @@
     <row r="156">
       <c r="A156" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">TH-TC-01</t>
+          <t xml:space="preserve">TH-INS-01</t>
         </is>
       </c>
       <c r="B156" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Tempco MTA1 custom ungrounded Type-K probes</t>
+          <t xml:space="preserve">secondary thermal barrier tape for grounded hot-shield exterior</t>
         </is>
       </c>
       <c r="C156" t="inlineStr" s="0">
@@ -13577,7 +13577,7 @@
       </c>
       <c r="E156" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">5</t>
+          <t xml:space="preserve">1</t>
         </is>
       </c>
       <c r="F156" t="inlineStr" s="0">
@@ -13587,12 +13587,12 @@
       </c>
       <c r="G156" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">BUY_TO_SPEC</t>
+          <t xml:space="preserve">MIXED</t>
         </is>
       </c>
       <c r="H156" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Alloy 600 MI sheath Ø3.00 ±0.03; 96% MgO; supplier-welded 304SS stop collar; process=buy/custom fabricate to thermal drawing note</t>
+          <t xml:space="preserve">received product; exact backing/adhesive/rating must be recorded</t>
         </is>
       </c>
       <c r="I156" t="inlineStr" s="0">
@@ -13617,12 +13617,12 @@
       </c>
       <c r="M156" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">USER_APPROVAL_AND_RECEIPT_TEST_HOLD</t>
+          <t xml:space="preserve">CANDIDATE_SELECTED—RECEIPT_TEST_REQUIRED</t>
         </is>
       </c>
       <c r="N156" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">exports/thermal/parts/TH-TC-01/drawing_notes.md</t>
+          <t xml:space="preserve">docs/drawings/v0.8/EX-003_heater_thermocouple.svg</t>
         </is>
       </c>
       <c r="O156" t="inlineStr" s="0">
@@ -13637,99 +13637,186 @@
       </c>
       <c r="Q156" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">SUBORDINATE DETAIL SOURCE: exports/thermal/manifest.csv; parent design authority remains bom/bom.csv; procurement/fabrication requires user approval</t>
+          <t xml:space="preserve">AUTHORITATIVE DESIGN SOURCE: bom/bom.csv; source=user stock; cash_class=REUSE_PENDING; status=RECEIPT_TEST_HOLD; quantity_unit=roll minimum; no safety function; no direct heater/barrel/die/cutoff/probe/terminal/vent coverage; S4 coupon smoke required; P9 adhesive-interface peak+U95+30 C must not exceed documented continuous rating; edge lift after cooldown &lt;=2 mm</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr" s="0">
         <is>
+          <t xml:space="preserve">TH-TC-01</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Tempco MTA1 custom ungrounded Type-K probes</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">final-design-fabrication-closure-v0.8</t>
+        </is>
+      </c>
+      <c r="D157" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">THERMAL</t>
+        </is>
+      </c>
+      <c r="E157" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">5</t>
+        </is>
+      </c>
+      <c r="F157" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">REQUIRED</t>
+        </is>
+      </c>
+      <c r="G157" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">BUY_TO_SPEC</t>
+        </is>
+      </c>
+      <c r="H157" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Alloy 600 MI sheath Ø3.00 ±0.03; 96% MgO; supplier-welded 304SS stop collar; process=buy/custom fabricate to thermal drawing note</t>
+        </is>
+      </c>
+      <c r="I157" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">heater fit, insulation, branch fuse and independent thermal cutoff</t>
+        </is>
+      </c>
+      <c r="J157" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">NONE_APPROVED—exact make/model and receipt evidence pending</t>
+        </is>
+      </c>
+      <c r="K157" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">NONE_APPROVED—deviation requires interface review and affected recalculation/calibration</t>
+        </is>
+      </c>
+      <c r="L157" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">NOT_APPLICABLE</t>
+        </is>
+      </c>
+      <c r="M157" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">USER_APPROVAL_AND_RECEIPT_TEST_HOLD</t>
+        </is>
+      </c>
+      <c r="N157" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">exports/thermal/parts/TH-TC-01/drawing_notes.md</t>
+        </is>
+      </c>
+      <c r="O157" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">docs/final/complete_build_manual_ko.pdf step 13; docs/final/assembly_steps.csv</t>
+        </is>
+      </c>
+      <c r="P157" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">firmware/arduino_mega/src + released pin map/calibration; physical calibration required</t>
+        </is>
+      </c>
+      <c r="Q157" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">SUBORDINATE DETAIL SOURCE: exports/thermal/manifest.csv; parent design authority remains bom/bom.csv; procurement/fabrication requires user approval</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr" s="0">
+        <is>
           <t xml:space="preserve">TH-TCR-01</t>
         </is>
       </c>
-      <c r="B157" t="inlineStr" s="0">
+      <c r="B158" t="inlineStr" s="0">
         <is>
           <t xml:space="preserve">Thermocouple stop-collar retainer bridge</t>
         </is>
       </c>
-      <c r="C157" t="inlineStr" s="0">
+      <c r="C158" t="inlineStr" s="0">
         <is>
           <t xml:space="preserve">final-design-fabrication-closure-v0.8</t>
         </is>
       </c>
-      <c r="D157" t="inlineStr" s="0">
+      <c r="D158" t="inlineStr" s="0">
         <is>
           <t xml:space="preserve">THERMAL</t>
         </is>
       </c>
-      <c r="E157" t="inlineStr" s="0">
+      <c r="E158" t="inlineStr" s="0">
         <is>
           <t xml:space="preserve">4</t>
         </is>
       </c>
-      <c r="F157" t="inlineStr" s="0">
+      <c r="F158" t="inlineStr" s="0">
         <is>
           <t xml:space="preserve">REQUIRED</t>
         </is>
       </c>
-      <c r="G157" t="inlineStr" s="0">
+      <c r="G158" t="inlineStr" s="0">
         <is>
           <t xml:space="preserve">BUY_TO_SPEC</t>
         </is>
       </c>
-      <c r="H157" t="inlineStr" s="0">
+      <c r="H158" t="inlineStr" s="0">
         <is>
           <t xml:space="preserve">304 stainless t1.5; process=buy/custom fabricate to thermal drawing note</t>
         </is>
       </c>
-      <c r="I157" t="inlineStr" s="0">
+      <c r="I158" t="inlineStr" s="0">
         <is>
           <t xml:space="preserve">heater fit, insulation, branch fuse and independent thermal cutoff</t>
         </is>
       </c>
-      <c r="J157" t="inlineStr" s="0">
+      <c r="J158" t="inlineStr" s="0">
         <is>
           <t xml:space="preserve">NONE_APPROVED—exact make/model and receipt evidence pending</t>
         </is>
       </c>
-      <c r="K157" t="inlineStr" s="0">
+      <c r="K158" t="inlineStr" s="0">
         <is>
           <t xml:space="preserve">NONE_APPROVED—deviation requires interface review and affected recalculation/calibration</t>
         </is>
       </c>
-      <c r="L157" t="inlineStr" s="0">
+      <c r="L158" t="inlineStr" s="0">
         <is>
           <t xml:space="preserve">NOT_APPLICABLE</t>
         </is>
       </c>
-      <c r="M157" t="inlineStr" s="0">
+      <c r="M158" t="inlineStr" s="0">
         <is>
           <t xml:space="preserve">USER_APPROVAL_AND_RECEIPT_TEST_HOLD</t>
         </is>
       </c>
-      <c r="N157" t="inlineStr" s="0">
+      <c r="N158" t="inlineStr" s="0">
         <is>
           <t xml:space="preserve">exports/thermal/parts/TH-TCR-01/drawing_notes.md</t>
         </is>
       </c>
-      <c r="O157" t="inlineStr" s="0">
+      <c r="O158" t="inlineStr" s="0">
         <is>
           <t xml:space="preserve">docs/final/complete_build_manual_ko.pdf step 13; docs/final/assembly_steps.csv</t>
         </is>
       </c>
-      <c r="P157" t="inlineStr" s="0">
+      <c r="P158" t="inlineStr" s="0">
         <is>
           <t xml:space="preserve">firmware/arduino_mega/src + released pin map/calibration; physical calibration required</t>
         </is>
       </c>
-      <c r="Q157" t="inlineStr" s="0">
+      <c r="Q158" t="inlineStr" s="0">
         <is>
           <t xml:space="preserve">SUBORDINATE DETAIL SOURCE: exports/thermal/manifest.csv; parent design authority remains bom/bom.csv; procurement/fabrication requires user approval</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Q157"/>
+  <autoFilter ref="A1:Q158"/>
 </worksheet>
 </file>
 
@@ -22249,78 +22336,115 @@
     <row r="156">
       <c r="A156" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">TH-TC-01</t>
+          <t xml:space="preserve">TH-INS-01</t>
         </is>
       </c>
       <c r="B156" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Tempco MTA1 custom ungrounded Type-K probes</t>
+          <t xml:space="preserve">secondary thermal barrier tape for grounded hot-shield exterior</t>
         </is>
       </c>
       <c r="C156" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">5</t>
+          <t xml:space="preserve">1</t>
         </is>
       </c>
       <c r="D156" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">BUY_TO_SPEC</t>
+          <t xml:space="preserve">MIXED</t>
         </is>
       </c>
       <c r="E156" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">SUBORDINATE DETAIL SOURCE: exports/thermal/manifest.csv</t>
+          <t xml:space="preserve">bom/bom.csv</t>
         </is>
       </c>
       <c r="F156" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">USER_APPROVAL_AND_RECEIPT_TEST_HOLD</t>
+          <t xml:space="preserve">CANDIDATE_SELECTED—RECEIPT_TEST_REQUIRED</t>
         </is>
       </c>
       <c r="G156" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Alloy 600 MI sheath Ø3.00 ±0.03; 96% MgO; supplier-welded 304SS stop collar; process=buy/custom fabricate to thermal drawing note</t>
+          <t xml:space="preserve">received product; exact backing/adhesive/rating must be recorded</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr" s="0">
         <is>
+          <t xml:space="preserve">TH-TC-01</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Tempco MTA1 custom ungrounded Type-K probes</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">5</t>
+        </is>
+      </c>
+      <c r="D157" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">BUY_TO_SPEC</t>
+        </is>
+      </c>
+      <c r="E157" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">SUBORDINATE DETAIL SOURCE: exports/thermal/manifest.csv</t>
+        </is>
+      </c>
+      <c r="F157" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">USER_APPROVAL_AND_RECEIPT_TEST_HOLD</t>
+        </is>
+      </c>
+      <c r="G157" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Alloy 600 MI sheath Ø3.00 ±0.03; 96% MgO; supplier-welded 304SS stop collar; process=buy/custom fabricate to thermal drawing note</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr" s="0">
+        <is>
           <t xml:space="preserve">TH-TCR-01</t>
         </is>
       </c>
-      <c r="B157" t="inlineStr" s="0">
+      <c r="B158" t="inlineStr" s="0">
         <is>
           <t xml:space="preserve">Thermocouple stop-collar retainer bridge</t>
         </is>
       </c>
-      <c r="C157" t="inlineStr" s="0">
+      <c r="C158" t="inlineStr" s="0">
         <is>
           <t xml:space="preserve">4</t>
         </is>
       </c>
-      <c r="D157" t="inlineStr" s="0">
+      <c r="D158" t="inlineStr" s="0">
         <is>
           <t xml:space="preserve">BUY_TO_SPEC</t>
         </is>
       </c>
-      <c r="E157" t="inlineStr" s="0">
+      <c r="E158" t="inlineStr" s="0">
         <is>
           <t xml:space="preserve">SUBORDINATE DETAIL SOURCE: exports/thermal/manifest.csv</t>
         </is>
       </c>
-      <c r="F157" t="inlineStr" s="0">
+      <c r="F158" t="inlineStr" s="0">
         <is>
           <t xml:space="preserve">USER_APPROVAL_AND_RECEIPT_TEST_HOLD</t>
         </is>
       </c>
-      <c r="G157" t="inlineStr" s="0">
+      <c r="G158" t="inlineStr" s="0">
         <is>
           <t xml:space="preserve">304 stainless t1.5; process=buy/custom fabricate to thermal drawing note</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G157"/>
+  <autoFilter ref="A1:G158"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
build(v0.8): regenerate PI tape-aware release artifacts
</commit_message>
<xml_diff>
--- a/exports/final/bom/BOM.xlsx
+++ b/exports/final/bom/BOM.xlsx
@@ -13562,7 +13562,7 @@
       </c>
       <c r="B156" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">secondary thermal barrier tape for grounded hot-shield exterior</t>
+          <t xml:space="preserve">PI gold finger polyimide thermal barrier tape, 25 mm x 30 m received roll</t>
         </is>
       </c>
       <c r="C156" t="inlineStr" s="0">
@@ -13592,7 +13592,7 @@
       </c>
       <c r="H156" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">received product; exact backing/adhesive/rating must be recorded</t>
+          <t xml:space="preserve">polyimide film; listing also states fluororesin release material; adhesive chemistry not specified</t>
         </is>
       </c>
       <c r="I156" t="inlineStr" s="0">
@@ -13637,7 +13637,7 @@
       </c>
       <c r="Q156" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">AUTHORITATIVE DESIGN SOURCE: bom/bom.csv; source=user stock; cash_class=REUSE_PENDING; status=RECEIPT_TEST_HOLD; quantity_unit=roll minimum; no safety function; no direct heater/barrel/die/cutoff/probe/terminal/vent coverage; S4 coupon smoke required; P9 adhesive-interface peak+U95+30 C must not exceed documented continuous rating; edge lift after cooldown &lt;=2 mm</t>
+          <t xml:space="preserve">AUTHORITATIVE DESIGN SOURCE: bom/bom.csv; source=user stock; cash_class=REUSE_PENDING; status=RECEIPT_TEST_HOLD; quantity_unit=each; received product claim long-term 220-280 C, short-term 300 C; use conservative 220 C continuous design basis; S4/P9 interface peak+U95 &lt;=190 C; no safety function; shield exterior only</t>
         </is>
       </c>
     </row>
@@ -22341,7 +22341,7 @@
       </c>
       <c r="B156" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">secondary thermal barrier tape for grounded hot-shield exterior</t>
+          <t xml:space="preserve">PI gold finger polyimide thermal barrier tape, 25 mm x 30 m received roll</t>
         </is>
       </c>
       <c r="C156" t="inlineStr" s="0">
@@ -22366,7 +22366,7 @@
       </c>
       <c r="G156" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">received product; exact backing/adhesive/rating must be recorded</t>
+          <t xml:space="preserve">polyimide film; listing also states fluororesin release material; adhesive chemistry not specified</t>
         </is>
       </c>
     </row>

</xml_diff>